<commit_message>
Curva Karol G v3 final: tallajes confirmados (tank tops y bikini S-L)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RmkPAi45jfkGpn6sh8ARUN
</commit_message>
<xml_diff>
--- a/produccion/Curva_Produccion_KarolG.xlsx
+++ b/produccion/Curva_Produccion_KarolG.xlsx
@@ -93,7 +93,7 @@
       <color rgb="00B91C1C"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -135,6 +135,11 @@
         <fgColor rgb="00DBEAFE"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DCFCE7"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -162,7 +167,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="46">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -216,6 +221,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -649,7 +657,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>KAROL G — Curva de producción final (v2: 9 referencias, mínimo 3.500 u)</t>
+          <t>KAROL G — Curva de producción final (v3 FINAL: 9 referencias, mínimo 3.500 u — tallajes confirmados 29-sep-2026)</t>
         </is>
       </c>
     </row>
@@ -1150,7 +1158,7 @@
       </c>
       <c r="B10" s="13" t="inlineStr">
         <is>
-          <t>S–XL (supuesto)</t>
+          <t>S–L</t>
         </is>
       </c>
       <c r="C10" s="14" t="inlineStr">
@@ -1230,7 +1238,7 @@
       </c>
       <c r="B11" s="13" t="inlineStr">
         <is>
-          <t>S–XL (supuesto)</t>
+          <t>S–L</t>
         </is>
       </c>
       <c r="C11" s="14" t="inlineStr">
@@ -1310,7 +1318,7 @@
       </c>
       <c r="B12" s="13" t="inlineStr">
         <is>
-          <t>S–L (supuesto)</t>
+          <t>S–L (conjunto)</t>
         </is>
       </c>
       <c r="C12" s="14" t="inlineStr">
@@ -2169,46 +2177,46 @@
       </c>
       <c r="B4" s="39" t="inlineStr">
         <is>
-          <t>Tallaje de tank tops y bikini</t>
+          <t>Unidades de referencias nuevas</t>
         </is>
       </c>
       <c r="C4" s="40" t="inlineStr">
         <is>
-          <t>No confirmado. Supuesto: tank tops S–XL (como la camiseta de tiras) y bikini S–L (XL es solo 3% de la venta histórica de bikinis). Confirmar antes de cortar.</t>
+          <t>Tank 180 + 180, bikini 160, pareo 130 son estimados sin historial Karol G (reparto aprobado por Mauricio 29-sep). Editables en "Parametros".</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="38" t="inlineStr">
-        <is>
-          <t>ALTA</t>
+      <c r="A5" s="41" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
         </is>
       </c>
       <c r="B5" s="39" t="inlineStr">
         <is>
-          <t>Unidades de referencias nuevas</t>
+          <t>Recorte a originales</t>
         </is>
       </c>
       <c r="C5" s="40" t="inlineStr">
         <is>
-          <t>Tank 180 + 180, bikini 160, pareo 130 son estimados sin historial Karol G. Editables en "Parametros"; el total se recalcula solo.</t>
+          <t>Las 5 referencias originales bajan 10% (3.204 → 2.890 u) para abrir espacio a las nuevas (aprobado).</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="38" t="inlineStr">
-        <is>
-          <t>ALTA</t>
+      <c r="A6" s="41" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
         </is>
       </c>
       <c r="B6" s="39" t="inlineStr">
         <is>
-          <t>Bikini = conjunto</t>
+          <t>Camisetas sin manga</t>
         </is>
       </c>
       <c r="C6" s="40" t="inlineStr">
         <is>
-          <t>Se asume 1 unidad = top + bottom de la misma talla. Si top y bottom se venden por separado, hay que partirlo en dos referencias con curva propia.</t>
+          <t>Camiseta de tiras + 2 tank tops = 900 u de un mismo tipo de prenda; riesgo de canibalización entre ellas.</t>
         </is>
       </c>
     </row>
@@ -2220,12 +2228,12 @@
       </c>
       <c r="B7" s="39" t="inlineStr">
         <is>
-          <t>Recorte a originales</t>
+          <t>Mesh manga larga</t>
         </is>
       </c>
       <c r="C7" s="40" t="inlineStr">
         <is>
-          <t>Las 5 referencias originales bajan 10% (3.204 → 2.890 u) para abrir espacio a las nuevas. Al subir el factor a 100% el grupo pasa a 3.854 u.</t>
+          <t>Usa solo el historial de mesh manga larga (167 u): muestra pequeña. La curva es casi igual a la de mesh long shirts (4.467 u).</t>
         </is>
       </c>
     </row>
@@ -2237,12 +2245,12 @@
       </c>
       <c r="B8" s="39" t="inlineStr">
         <is>
-          <t>Camisetas sin manga</t>
+          <t>Solo canal Shopify</t>
         </is>
       </c>
       <c r="C8" s="40" t="inlineStr">
         <is>
-          <t>Camiseta de tiras + 2 tank tops = 900 u de un mismo tipo de prenda; riesgo de canibalización entre ellas.</t>
+          <t>El historial no incluye mayoristas ni exportación. Un pedido mayorista de Karol G debe sumar su curva aparte.</t>
         </is>
       </c>
     </row>
@@ -2254,12 +2262,12 @@
       </c>
       <c r="B9" s="39" t="inlineStr">
         <is>
-          <t>Mesh manga larga</t>
+          <t>Unidades pequeñas en extremos</t>
         </is>
       </c>
       <c r="C9" s="40" t="inlineStr">
         <is>
-          <t>Ahora usa solo el historial de mesh manga larga (167 u): muestra pequeña. La curva es casi igual a la de mesh long shirts (4.467 u).</t>
+          <t>Varias tallas XS/XL y la L del bikini quedan con menos de 60 u; validar mínimos por corte con el satélite.</t>
         </is>
       </c>
     </row>
@@ -2271,12 +2279,12 @@
       </c>
       <c r="B10" s="39" t="inlineStr">
         <is>
-          <t>Solo canal Shopify</t>
+          <t>Bikini: top y bottom</t>
         </is>
       </c>
       <c r="C10" s="40" t="inlineStr">
         <is>
-          <t>El historial no incluye mayoristas ni exportación. Un pedido mayorista de Karol G debe sumar su curva aparte.</t>
+          <t>Se vende como conjunto: producir top y bottom en la misma cantidad por talla (160 conjuntos = 160 tops + 160 bottoms).</t>
         </is>
       </c>
     </row>
@@ -2288,46 +2296,46 @@
       </c>
       <c r="B11" s="39" t="inlineStr">
         <is>
-          <t>Unidades pequeñas en extremos</t>
+          <t>Insumos de Jean y collares</t>
         </is>
       </c>
       <c r="C11" s="40" t="inlineStr">
         <is>
-          <t>Varias tallas XS/XL quedan con menos de 60 u; validar mínimos por corte con el satélite.</t>
+          <t>Si ya se compró o separó tela o herrajes para Jean y collares (720 u), cancelar o reasignar.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="41" t="inlineStr">
-        <is>
-          <t>MEDIA</t>
+      <c r="A12" s="42" t="inlineStr">
+        <is>
+          <t>INFO</t>
         </is>
       </c>
       <c r="B12" s="39" t="inlineStr">
         <is>
-          <t>Insumos de Jean y collares</t>
+          <t>Tiempos</t>
         </is>
       </c>
       <c r="C12" s="40" t="inlineStr">
         <is>
-          <t>Si ya se compró o separó tela o herrajes para Jean y collares (720 u), cancelar o reasignar (¿al bikini/pareo?).</t>
+          <t>4 referencias nuevas requieren patronaje/muestra. Confirmar fecha compromiso del satélite para fin de año.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="42" t="inlineStr">
-        <is>
-          <t>INFO</t>
+      <c r="A13" s="43" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
       <c r="B13" s="39" t="inlineStr">
         <is>
-          <t>Tiempos</t>
+          <t>Tallajes confirmados</t>
         </is>
       </c>
       <c r="C13" s="40" t="inlineStr">
         <is>
-          <t>Correo original del 14-sep; se agregan 4 referencias nuevas que necesitan patronaje/muestra. Confirmar fecha compromiso del satélite para fin de año.</t>
+          <t>Camiseta de tiras S–XL, Body negro S–XL, Tank tops S–L, Bikini S–L (conjunto), Mesh = manga larga, 1 color por referencia.</t>
         </is>
       </c>
     </row>
@@ -2428,25 +2436,25 @@
           <t>T-shirts Mompossina sin Colombia, renormalizado a S–XL (tallaje confirmado)</t>
         </is>
       </c>
-      <c r="C5" s="43" t="n">
+      <c r="C5" s="44" t="n">
         <v>0</v>
       </c>
-      <c r="D5" s="43" t="n">
+      <c r="D5" s="44" t="n">
         <v>415</v>
       </c>
-      <c r="E5" s="43" t="n">
+      <c r="E5" s="44" t="n">
         <v>614</v>
       </c>
-      <c r="F5" s="43" t="n">
+      <c r="F5" s="44" t="n">
         <v>290</v>
       </c>
-      <c r="G5" s="43" t="n">
+      <c r="G5" s="44" t="n">
         <v>155</v>
       </c>
-      <c r="H5" s="43" t="n">
+      <c r="H5" s="44" t="n">
         <v>0</v>
       </c>
-      <c r="I5" s="44">
+      <c r="I5" s="45">
         <f>SUM(C5:H5)</f>
         <v/>
       </c>
@@ -2462,25 +2470,25 @@
           <t>Mesh shirts manga corta (sin Colombia Mesh Shirt)</t>
         </is>
       </c>
-      <c r="C6" s="43" t="n">
+      <c r="C6" s="44" t="n">
         <v>324</v>
       </c>
-      <c r="D6" s="43" t="n">
+      <c r="D6" s="44" t="n">
         <v>1090</v>
       </c>
-      <c r="E6" s="43" t="n">
+      <c r="E6" s="44" t="n">
         <v>1403</v>
       </c>
-      <c r="F6" s="43" t="n">
+      <c r="F6" s="44" t="n">
         <v>839</v>
       </c>
-      <c r="G6" s="43" t="n">
+      <c r="G6" s="44" t="n">
         <v>392</v>
       </c>
-      <c r="H6" s="43" t="n">
+      <c r="H6" s="44" t="n">
         <v>0</v>
       </c>
-      <c r="I6" s="44">
+      <c r="I6" s="45">
         <f>SUM(C6:H6)</f>
         <v/>
       </c>
@@ -2496,25 +2504,25 @@
           <t>Todos los bodies (tallaje S–XL confirmado)</t>
         </is>
       </c>
-      <c r="C7" s="43" t="n">
+      <c r="C7" s="44" t="n">
         <v>0</v>
       </c>
-      <c r="D7" s="43" t="n">
+      <c r="D7" s="44" t="n">
         <v>217</v>
       </c>
-      <c r="E7" s="43" t="n">
+      <c r="E7" s="44" t="n">
         <v>240</v>
       </c>
-      <c r="F7" s="43" t="n">
+      <c r="F7" s="44" t="n">
         <v>166</v>
       </c>
-      <c r="G7" s="43" t="n">
+      <c r="G7" s="44" t="n">
         <v>73</v>
       </c>
-      <c r="H7" s="43" t="n">
+      <c r="H7" s="44" t="n">
         <v>0</v>
       </c>
-      <c r="I7" s="44">
+      <c r="I7" s="45">
         <f>SUM(C7:H7)</f>
         <v/>
       </c>
@@ -2530,25 +2538,25 @@
           <t>Mesh LONG SLEEVE shirts (I'm Black / I'm White) — manga larga confirmada</t>
         </is>
       </c>
-      <c r="C8" s="43" t="n">
+      <c r="C8" s="44" t="n">
         <v>11</v>
       </c>
-      <c r="D8" s="43" t="n">
+      <c r="D8" s="44" t="n">
         <v>50</v>
       </c>
-      <c r="E8" s="43" t="n">
+      <c r="E8" s="44" t="n">
         <v>57</v>
       </c>
-      <c r="F8" s="43" t="n">
+      <c r="F8" s="44" t="n">
         <v>31</v>
       </c>
-      <c r="G8" s="43" t="n">
+      <c r="G8" s="44" t="n">
         <v>18</v>
       </c>
-      <c r="H8" s="43" t="n">
+      <c r="H8" s="44" t="n">
         <v>0</v>
       </c>
-      <c r="I8" s="44">
+      <c r="I8" s="45">
         <f>SUM(C8:H8)</f>
         <v/>
       </c>
@@ -2564,25 +2572,25 @@
           <t>T-shirts Mompossina (sin Colombia T-shirt)</t>
         </is>
       </c>
-      <c r="C9" s="43" t="n">
+      <c r="C9" s="44" t="n">
         <v>162</v>
       </c>
-      <c r="D9" s="43" t="n">
+      <c r="D9" s="44" t="n">
         <v>415</v>
       </c>
-      <c r="E9" s="43" t="n">
+      <c r="E9" s="44" t="n">
         <v>614</v>
       </c>
-      <c r="F9" s="43" t="n">
+      <c r="F9" s="44" t="n">
         <v>290</v>
       </c>
-      <c r="G9" s="43" t="n">
+      <c r="G9" s="44" t="n">
         <v>155</v>
       </c>
-      <c r="H9" s="43" t="n">
+      <c r="H9" s="44" t="n">
         <v>0</v>
       </c>
-      <c r="I9" s="44">
+      <c r="I9" s="45">
         <f>SUM(C9:H9)</f>
         <v/>
       </c>
@@ -2595,28 +2603,28 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>T-shirts S–XL (el único tank histórico, Amor Tank Top, 96 u, solo S/M/L)</t>
-        </is>
-      </c>
-      <c r="C10" s="43" t="n">
+          <t>Amor Tank Top (96 u) + T-shirts sin Colombia, solo S–L (tallaje confirmado)</t>
+        </is>
+      </c>
+      <c r="C10" s="44" t="n">
         <v>0</v>
       </c>
-      <c r="D10" s="43" t="n">
-        <v>415</v>
-      </c>
-      <c r="E10" s="43" t="n">
-        <v>614</v>
-      </c>
-      <c r="F10" s="43" t="n">
-        <v>290</v>
-      </c>
-      <c r="G10" s="43" t="n">
-        <v>155</v>
-      </c>
-      <c r="H10" s="43" t="n">
+      <c r="D10" s="44" t="n">
+        <v>443</v>
+      </c>
+      <c r="E10" s="44" t="n">
+        <v>656</v>
+      </c>
+      <c r="F10" s="44" t="n">
+        <v>316</v>
+      </c>
+      <c r="G10" s="44" t="n">
         <v>0</v>
       </c>
-      <c r="I10" s="44">
+      <c r="H10" s="44" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" s="45">
         <f>SUM(C10:H10)</f>
         <v/>
       </c>
@@ -2629,28 +2637,28 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>T-shirts S–XL (el único tank histórico, Amor Tank Top, 96 u, solo S/M/L)</t>
-        </is>
-      </c>
-      <c r="C11" s="43" t="n">
+          <t>Amor Tank Top (96 u) + T-shirts sin Colombia, solo S–L (tallaje confirmado)</t>
+        </is>
+      </c>
+      <c r="C11" s="44" t="n">
         <v>0</v>
       </c>
-      <c r="D11" s="43" t="n">
-        <v>415</v>
-      </c>
-      <c r="E11" s="43" t="n">
-        <v>614</v>
-      </c>
-      <c r="F11" s="43" t="n">
-        <v>290</v>
-      </c>
-      <c r="G11" s="43" t="n">
-        <v>155</v>
-      </c>
-      <c r="H11" s="43" t="n">
+      <c r="D11" s="44" t="n">
+        <v>443</v>
+      </c>
+      <c r="E11" s="44" t="n">
+        <v>656</v>
+      </c>
+      <c r="F11" s="44" t="n">
+        <v>316</v>
+      </c>
+      <c r="G11" s="44" t="n">
         <v>0</v>
       </c>
-      <c r="I11" s="44">
+      <c r="H11" s="44" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" s="45">
         <f>SUM(C11:H11)</f>
         <v/>
       </c>
@@ -2663,28 +2671,28 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>Tops de bikini + bottoms Mompossina (XL = 3% histórico, se omite)</t>
-        </is>
-      </c>
-      <c r="C12" s="43" t="n">
+          <t>Tops de bikini + bottoms Mompossina, S–L (tallaje confirmado; se vende como conjunto)</t>
+        </is>
+      </c>
+      <c r="C12" s="44" t="n">
         <v>0</v>
       </c>
-      <c r="D12" s="43" t="n">
+      <c r="D12" s="44" t="n">
         <v>864</v>
       </c>
-      <c r="E12" s="43" t="n">
+      <c r="E12" s="44" t="n">
         <v>1434</v>
       </c>
-      <c r="F12" s="43" t="n">
+      <c r="F12" s="44" t="n">
         <v>733</v>
       </c>
-      <c r="G12" s="43" t="n">
+      <c r="G12" s="44" t="n">
         <v>0</v>
       </c>
-      <c r="H12" s="43" t="n">
+      <c r="H12" s="44" t="n">
         <v>0</v>
       </c>
-      <c r="I12" s="44">
+      <c r="I12" s="45">
         <f>SUM(C12:H12)</f>
         <v/>
       </c>
@@ -2700,25 +2708,25 @@
           <t>Talla única</t>
         </is>
       </c>
-      <c r="C13" s="43" t="n">
+      <c r="C13" s="44" t="n">
         <v>0</v>
       </c>
-      <c r="D13" s="43" t="n">
+      <c r="D13" s="44" t="n">
         <v>0</v>
       </c>
-      <c r="E13" s="43" t="n">
+      <c r="E13" s="44" t="n">
         <v>0</v>
       </c>
-      <c r="F13" s="43" t="n">
+      <c r="F13" s="44" t="n">
         <v>0</v>
       </c>
-      <c r="G13" s="43" t="n">
+      <c r="G13" s="44" t="n">
         <v>0</v>
       </c>
-      <c r="H13" s="43" t="n">
+      <c r="H13" s="44" t="n">
         <v>1</v>
       </c>
-      <c r="I13" s="44">
+      <c r="I13" s="45">
         <f>SUM(C13:H13)</f>
         <v/>
       </c>

</xml_diff>